<commit_message>
Update listedness: Apixaban / Metamorphopsia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2003"/>
+  <dimension ref="A1:D2004"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36774,6 +36774,24 @@
       </c>
       <c r="D2003" t="inlineStr"/>
     </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>Metamorphopsia</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2004" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: FAMOTIDINE / Dyschromatopsia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2004"/>
+  <dimension ref="A1:D2005"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36792,6 +36792,24 @@
       </c>
       <c r="D2004" t="inlineStr"/>
     </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>FAMOTIDINE</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>Dyschromatopsia</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2005" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Hyperhidrosis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2005"/>
+  <dimension ref="A1:D2006"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36810,6 +36810,24 @@
       </c>
       <c r="D2005" t="inlineStr"/>
     </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>Hyperhidrosis</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2006" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Cerebrovascular accident
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2006"/>
+  <dimension ref="A1:D2007"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36828,6 +36828,24 @@
       </c>
       <c r="D2006" t="inlineStr"/>
     </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>Cerebrovascular accident</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2007" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APREMILAST / Product ineffective
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2007"/>
+  <dimension ref="A1:D2008"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36846,6 +36846,24 @@
       </c>
       <c r="D2007" t="inlineStr"/>
     </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>Product ineffective</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2008" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Anal haemorrhage
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2008"/>
+  <dimension ref="A1:D2009"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36864,6 +36864,24 @@
       </c>
       <c r="D2008" t="inlineStr"/>
     </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>Anal haemorrhage</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2009" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Sinus headache
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2009"/>
+  <dimension ref="A1:D2010"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36882,6 +36882,24 @@
       </c>
       <c r="D2009" t="inlineStr"/>
     </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>Sinus headache</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2010" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: Clobazam / Epilepsy
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2010"/>
+  <dimension ref="A1:D2011"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36900,6 +36900,24 @@
       </c>
       <c r="D2010" t="inlineStr"/>
     </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>CLOBAZAM</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>Epilepsy</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2011" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: Clobazam / Hospitalisation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2011"/>
+  <dimension ref="A1:D2012"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36918,6 +36918,24 @@
       </c>
       <c r="D2011" t="inlineStr"/>
     </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>CLOBAZAM</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>Hospitalisation</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2012" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: Clobazam / Illness
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2012"/>
+  <dimension ref="A1:D2013"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36936,6 +36936,24 @@
       </c>
       <c r="D2012" t="inlineStr"/>
     </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>CLOBAZAM</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>Illness</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2013" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: Clobazam / Adverse event
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2013"/>
+  <dimension ref="A1:D2014"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36954,6 +36954,24 @@
       </c>
       <c r="D2013" t="inlineStr"/>
     </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>CLOBAZAM</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>Adverse event</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2014" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Osteoarthritis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2014"/>
+  <dimension ref="A1:D2015"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36972,6 +36972,24 @@
       </c>
       <c r="D2014" t="inlineStr"/>
     </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>Osteoarthritis</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2015" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Adverse drug reaction
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2015"/>
+  <dimension ref="A1:D2016"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -36990,6 +36990,24 @@
       </c>
       <c r="D2015" t="inlineStr"/>
     </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>Adverse drug reaction</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2016" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Subdural haematoma
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2016"/>
+  <dimension ref="A1:D2017"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37008,6 +37008,24 @@
       </c>
       <c r="D2016" t="inlineStr"/>
     </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>Subdural haematoma</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2017" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APREMILAST / Dizziness
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2017"/>
+  <dimension ref="A1:D2018"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37026,6 +37026,24 @@
       </c>
       <c r="D2017" t="inlineStr"/>
     </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>Dizziness</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2018" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Adverse drug reaction
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2018"/>
+  <dimension ref="A1:D2019"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37044,6 +37044,24 @@
       </c>
       <c r="D2018" t="inlineStr"/>
     </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>Adverse drug reaction</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2019" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Ketosis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2019"/>
+  <dimension ref="A1:D2020"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37062,6 +37062,24 @@
       </c>
       <c r="D2019" t="inlineStr"/>
     </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>Ketosis</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2020" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Blister
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2020"/>
+  <dimension ref="A1:D2021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37080,6 +37080,24 @@
       </c>
       <c r="D2020" t="inlineStr"/>
     </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>Blister</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2021" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Cellulitis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2021"/>
+  <dimension ref="A1:D2022"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37098,6 +37098,24 @@
       </c>
       <c r="D2021" t="inlineStr"/>
     </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>Cellulitis</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2022" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Sepsis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2022"/>
+  <dimension ref="A1:D2023"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37116,6 +37116,24 @@
       </c>
       <c r="D2022" t="inlineStr"/>
     </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>Sepsis</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2023" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Pemphigoid
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2023"/>
+  <dimension ref="A1:D2024"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37134,6 +37134,24 @@
       </c>
       <c r="D2023" t="inlineStr"/>
     </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>Pemphigoid</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2024" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Knee operation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2024"/>
+  <dimension ref="A1:D2025"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37152,6 +37152,24 @@
       </c>
       <c r="D2024" t="inlineStr"/>
     </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>Knee operation</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2025" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: CLONAZEPAM / Chest pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2025"/>
+  <dimension ref="A1:D2026"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37170,6 +37170,24 @@
       </c>
       <c r="D2025" t="inlineStr"/>
     </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>CLONAZEPAM</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>Chest pain</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2026" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Erythema
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2026"/>
+  <dimension ref="A1:D2027"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37188,6 +37188,24 @@
       </c>
       <c r="D2026" t="inlineStr"/>
     </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>Erythema</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2027" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Faeces soft
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2027"/>
+  <dimension ref="A1:D2028"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37206,6 +37206,24 @@
       </c>
       <c r="D2027" t="inlineStr"/>
     </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>Faeces soft</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2028" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Aggression
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2028"/>
+  <dimension ref="A1:D2029"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37224,6 +37224,24 @@
       </c>
       <c r="D2028" t="inlineStr"/>
     </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>Aggression</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2029" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Drug eruption
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2029"/>
+  <dimension ref="A1:D2030"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37242,6 +37242,24 @@
       </c>
       <c r="D2029" t="inlineStr"/>
     </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>Drug eruption</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2030" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Taste disorder
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2030"/>
+  <dimension ref="A1:D2031"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37260,6 +37260,24 @@
       </c>
       <c r="D2030" t="inlineStr"/>
     </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>Taste disorder</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2031" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Protein total
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2031"/>
+  <dimension ref="A1:D2032"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37278,6 +37278,24 @@
       </c>
       <c r="D2031" t="inlineStr"/>
     </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>Protein total</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2032" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Anxiety
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2032"/>
+  <dimension ref="A1:D2033"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37296,6 +37296,24 @@
       </c>
       <c r="D2032" t="inlineStr"/>
     </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>Anxiety</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2033" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Depression
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2033"/>
+  <dimension ref="A1:D2034"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37314,6 +37314,24 @@
       </c>
       <c r="D2033" t="inlineStr"/>
     </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>Depression</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2034" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Hypoaesthesia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2034"/>
+  <dimension ref="A1:D2035"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37332,6 +37332,24 @@
       </c>
       <c r="D2034" t="inlineStr"/>
     </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>Hypoaesthesia</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2035" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Disease progression
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2035"/>
+  <dimension ref="A1:D2036"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37350,6 +37350,24 @@
       </c>
       <c r="D2035" t="inlineStr"/>
     </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>Disease progression</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2036" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Chest discomfort
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2036"/>
+  <dimension ref="A1:D2037"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37368,6 +37368,24 @@
       </c>
       <c r="D2036" t="inlineStr"/>
     </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>Chest discomfort</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2037" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Erythema
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2037"/>
+  <dimension ref="A1:D2038"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37386,6 +37386,24 @@
       </c>
       <c r="D2037" t="inlineStr"/>
     </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>Erythema</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2038" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Urinary tract candidiasis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2038"/>
+  <dimension ref="A1:D2039"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37404,6 +37404,24 @@
       </c>
       <c r="D2038" t="inlineStr"/>
     </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>Urinary tract candidiasis</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2039" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Cyanosis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2039"/>
+  <dimension ref="A1:D2040"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37422,6 +37422,24 @@
       </c>
       <c r="D2039" t="inlineStr"/>
     </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>Cyanosis</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2040" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Retroperitoneal haematoma
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2040"/>
+  <dimension ref="A1:D2041"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37440,6 +37440,24 @@
       </c>
       <c r="D2040" t="inlineStr"/>
     </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>Retroperitoneal haematoma</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2041" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Renal artery thrombosis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2041"/>
+  <dimension ref="A1:D2042"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37458,6 +37458,24 @@
       </c>
       <c r="D2041" t="inlineStr"/>
     </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>Renal artery thrombosis</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2042" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Renal colic
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2042"/>
+  <dimension ref="A1:D2043"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37476,6 +37476,24 @@
       </c>
       <c r="D2042" t="inlineStr"/>
     </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>Renal colic</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2043" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Renal pseudoaneurysm
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2043"/>
+  <dimension ref="A1:D2044"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37494,6 +37494,24 @@
       </c>
       <c r="D2043" t="inlineStr"/>
     </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>Renal pseudoaneurysm</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2044" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Parosmia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2044"/>
+  <dimension ref="A1:D2045"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37512,6 +37512,24 @@
       </c>
       <c r="D2044" t="inlineStr"/>
     </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>Parosmia</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2045" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Pemphigoid
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2045"/>
+  <dimension ref="A1:D2046"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37530,6 +37530,24 @@
       </c>
       <c r="D2045" t="inlineStr"/>
     </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>Pemphigoid</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2046" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RANOLAZINE / Rash erythematous
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2046"/>
+  <dimension ref="A1:D2047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37548,6 +37548,24 @@
       </c>
       <c r="D2046" t="inlineStr"/>
     </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>RANOLAZINE</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>Rash erythematous</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2047" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RANOLAZINE / Swelling face
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2047"/>
+  <dimension ref="A1:D2048"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37566,6 +37566,24 @@
       </c>
       <c r="D2047" t="inlineStr"/>
     </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>RANOLAZINE</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>Swelling face</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2048" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Pain in jaw
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2048"/>
+  <dimension ref="A1:D2049"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37584,6 +37584,24 @@
       </c>
       <c r="D2048" t="inlineStr"/>
     </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>Pain in jaw</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2049" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Drug ineffective
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2049"/>
+  <dimension ref="A1:D2050"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37602,6 +37602,24 @@
       </c>
       <c r="D2049" t="inlineStr"/>
     </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>Drug ineffective</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2050" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SAFINAMIDE / Nausea
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2050"/>
+  <dimension ref="A1:D2051"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37620,6 +37620,24 @@
       </c>
       <c r="D2050" t="inlineStr"/>
     </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>SAFINAMIDE</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>Nausea</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2051" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Sinus bradycardia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2051"/>
+  <dimension ref="A1:D2052"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37638,6 +37638,24 @@
       </c>
       <c r="D2051" t="inlineStr"/>
     </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>Sinus bradycardia</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2052" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: BRIVARACETAM / Dermatitis allergic
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2052"/>
+  <dimension ref="A1:D2053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37656,6 +37656,24 @@
       </c>
       <c r="D2052" t="inlineStr"/>
     </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>BRIVARACETAM</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>Dermatitis allergic</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2053" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: BRIVARACETAM / Sedation complication
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2053"/>
+  <dimension ref="A1:D2054"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37674,6 +37674,24 @@
       </c>
       <c r="D2053" t="inlineStr"/>
     </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>BRIVARACETAM</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>Sedation complication</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2054" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Pollakiuria
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2054"/>
+  <dimension ref="A1:D2055"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37692,6 +37692,24 @@
       </c>
       <c r="D2054" t="inlineStr"/>
     </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>Pollakiuria</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2055" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: SITAGLIPTIN / Renal pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2055"/>
+  <dimension ref="A1:D2056"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37710,6 +37710,24 @@
       </c>
       <c r="D2055" t="inlineStr"/>
     </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>SITAGLIPTIN</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>Renal pain</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2056" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: BRIVARACETAM / Headache
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2056"/>
+  <dimension ref="A1:D2057"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37728,6 +37728,24 @@
       </c>
       <c r="D2056" t="inlineStr"/>
     </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>BRIVARACETAM</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>Headache</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2057" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Accelerated hypertension
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2057"/>
+  <dimension ref="A1:D2058"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37746,6 +37746,24 @@
       </c>
       <c r="D2057" t="inlineStr"/>
     </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>Accelerated hypertension</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2058" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Mood swings
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2058"/>
+  <dimension ref="A1:D2059"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37764,6 +37764,24 @@
       </c>
       <c r="D2058" t="inlineStr"/>
     </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>Mood swings</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2059" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Vulvovaginal inflammation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2059"/>
+  <dimension ref="A1:D2060"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37782,6 +37782,24 @@
       </c>
       <c r="D2059" t="inlineStr"/>
     </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>Vulvovaginal inflammation</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2060" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Blood urine present
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2060"/>
+  <dimension ref="A1:D2061"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37800,6 +37800,24 @@
       </c>
       <c r="D2060" t="inlineStr"/>
     </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>Blood urine present</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2061" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Burning sensation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2061"/>
+  <dimension ref="A1:D2062"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37818,6 +37818,24 @@
       </c>
       <c r="D2061" t="inlineStr"/>
     </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>Burning sensation</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2062" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Aphthous ulcer
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2062"/>
+  <dimension ref="A1:D2063"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37836,6 +37836,24 @@
       </c>
       <c r="D2062" t="inlineStr"/>
     </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>Aphthous ulcer</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2063" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Disorientation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2063"/>
+  <dimension ref="A1:D2064"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37854,6 +37854,24 @@
       </c>
       <c r="D2063" t="inlineStr"/>
     </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>Disorientation</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2064" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Faeces hard
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2064"/>
+  <dimension ref="A1:D2065"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37872,6 +37872,24 @@
       </c>
       <c r="D2064" t="inlineStr"/>
     </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>Faeces hard</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2065" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Toe operation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2065"/>
+  <dimension ref="A1:D2066"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37890,6 +37890,24 @@
       </c>
       <c r="D2065" t="inlineStr"/>
     </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>Toe operation</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2066" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Product colour issue
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2066"/>
+  <dimension ref="A1:D2067"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37908,6 +37908,24 @@
       </c>
       <c r="D2066" t="inlineStr"/>
     </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>Product colour issue</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2067" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Product with quality issue administered
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2067"/>
+  <dimension ref="A1:D2068"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37926,6 +37926,24 @@
       </c>
       <c r="D2067" t="inlineStr"/>
     </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>Product with quality issue administered</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2068" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: BRIVARACETAM / Suicidal behaviour
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2068"/>
+  <dimension ref="A1:D2069"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37944,6 +37944,24 @@
       </c>
       <c r="D2068" t="inlineStr"/>
     </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>BRIVARACETAM</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>Suicidal behaviour</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2069" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Flat affect
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2069"/>
+  <dimension ref="A1:D2070"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37962,6 +37962,24 @@
       </c>
       <c r="D2069" t="inlineStr"/>
     </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>Flat affect</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2070" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Gastroenteritis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2070"/>
+  <dimension ref="A1:D2071"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37980,6 +37980,24 @@
       </c>
       <c r="D2070" t="inlineStr"/>
     </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>Gastroenteritis</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2071" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Adverse drug reaction
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2071"/>
+  <dimension ref="A1:D2072"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37998,6 +37998,24 @@
       </c>
       <c r="D2071" t="inlineStr"/>
     </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>Adverse drug reaction</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2072" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Glossodynia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2072"/>
+  <dimension ref="A1:D2073"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38016,6 +38016,24 @@
       </c>
       <c r="D2072" t="inlineStr"/>
     </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>Glossodynia</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2073" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Hyperhidrosis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2073"/>
+  <dimension ref="A1:D2074"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38034,6 +38034,24 @@
       </c>
       <c r="D2073" t="inlineStr"/>
     </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>Hyperhidrosis</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2074" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Contusion
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2074"/>
+  <dimension ref="A1:D2075"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38052,6 +38052,24 @@
       </c>
       <c r="D2074" t="inlineStr"/>
     </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>Contusion</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2075" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Disorientation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2075"/>
+  <dimension ref="A1:D2076"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38070,6 +38070,24 @@
       </c>
       <c r="D2075" t="inlineStr"/>
     </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>Disorientation</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2076" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Incontinence
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2076"/>
+  <dimension ref="A1:D2077"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38088,6 +38088,24 @@
       </c>
       <c r="D2076" t="inlineStr"/>
     </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>Incontinence</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2077" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Hospitalisation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2077"/>
+  <dimension ref="A1:D2078"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38106,6 +38106,24 @@
       </c>
       <c r="D2077" t="inlineStr"/>
     </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>Hospitalisation</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2078" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2078"/>
+  <dimension ref="A1:D2079"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38124,6 +38124,24 @@
       </c>
       <c r="D2078" t="inlineStr"/>
     </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2079" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Renal pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2079"/>
+  <dimension ref="A1:D2080"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38142,6 +38142,24 @@
       </c>
       <c r="D2079" t="inlineStr"/>
     </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>Renal pain</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2080" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Brain fog
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2080"/>
+  <dimension ref="A1:D2081"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38160,6 +38160,24 @@
       </c>
       <c r="D2080" t="inlineStr"/>
     </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>Brain fog</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2081" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Exposure during pregnancy
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2081"/>
+  <dimension ref="A1:D2082"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38178,6 +38178,24 @@
       </c>
       <c r="D2081" t="inlineStr"/>
     </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>Exposure during pregnancy</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2082" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Paraesthesia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2082"/>
+  <dimension ref="A1:D2083"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38196,6 +38196,24 @@
       </c>
       <c r="D2082" t="inlineStr"/>
     </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>Paraesthesia</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2083" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Aggression
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2083"/>
+  <dimension ref="A1:D2084"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38214,6 +38214,24 @@
       </c>
       <c r="D2083" t="inlineStr"/>
     </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>Aggression</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2084" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Heart rate irregular
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2084"/>
+  <dimension ref="A1:D2085"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38232,6 +38232,24 @@
       </c>
       <c r="D2084" t="inlineStr"/>
     </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>Heart rate irregular</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2085" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch update listedness: 0 added, 1 updated
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -1894,7 +1894,11 @@
           <t>Unexpected</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Dizziness with Cerebral haemorrhage should be considered as Listed</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">

</xml_diff>

<commit_message>
Batch update listedness: 2 added, 5 updated
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2085"/>
+  <dimension ref="A1:D2087"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38254,6 +38254,42 @@
       </c>
       <c r="D2085" t="inlineStr"/>
     </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>Cauda equina syndrome</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2086" t="inlineStr"/>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>Spinal subdural haematoma</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2087" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Suprapubic pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2087"/>
+  <dimension ref="A1:D2088"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38290,6 +38290,24 @@
       </c>
       <c r="D2087" t="inlineStr"/>
     </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>Suprapubic pain</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2088" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: BRIVARACETAM / Somnambulism
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2088"/>
+  <dimension ref="A1:D2089"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38308,6 +38308,24 @@
       </c>
       <c r="D2088" t="inlineStr"/>
     </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>BRIVARACETAM</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>Somnambulism</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2089" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Depressed mood
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2089"/>
+  <dimension ref="A1:D2090"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38326,6 +38326,24 @@
       </c>
       <c r="D2089" t="inlineStr"/>
     </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>Depressed mood</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2090" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Bladder pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2090"/>
+  <dimension ref="A1:D2091"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38344,6 +38344,24 @@
       </c>
       <c r="D2090" t="inlineStr"/>
     </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>Bladder pain</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2091" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Vulvovaginal burning sensation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2091"/>
+  <dimension ref="A1:D2092"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38362,6 +38362,24 @@
       </c>
       <c r="D2091" t="inlineStr"/>
     </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>Vulvovaginal burning sensation</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2092" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Urethral pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2092"/>
+  <dimension ref="A1:D2093"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38380,6 +38380,24 @@
       </c>
       <c r="D2092" t="inlineStr"/>
     </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>Urethral pain</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2093" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APREMILAST / Abdominal discomfort
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2093"/>
+  <dimension ref="A1:D2094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38398,6 +38398,24 @@
       </c>
       <c r="D2093" t="inlineStr"/>
     </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr">
+        <is>
+          <t>Abdominal discomfort</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2094" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Fungaemia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2094"/>
+  <dimension ref="A1:D2095"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38416,6 +38416,24 @@
       </c>
       <c r="D2094" t="inlineStr"/>
     </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>Fungaemia</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2095" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Dairy intolerance
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2095"/>
+  <dimension ref="A1:D2096"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38434,6 +38434,24 @@
       </c>
       <c r="D2095" t="inlineStr"/>
     </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr">
+        <is>
+          <t>Dairy intolerance</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2096" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Dry eye
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2096"/>
+  <dimension ref="A1:D2097"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38452,6 +38452,24 @@
       </c>
       <c r="D2096" t="inlineStr"/>
     </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>Dry eye</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2097" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Septic shock
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2097"/>
+  <dimension ref="A1:D2098"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38470,6 +38470,28 @@
       </c>
       <c r="D2097" t="inlineStr"/>
     </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr">
+        <is>
+          <t>Septic shock</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2098" t="inlineStr">
+        <is>
+          <t>Expected along with Fournier's Gangrene</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APIXABAN / Tooth extraction
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2098"/>
+  <dimension ref="A1:D2099"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38492,6 +38492,24 @@
         </is>
       </c>
     </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>APIXABAN</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>Tooth extraction</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2099" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Product formulation issue
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2099"/>
+  <dimension ref="A1:D2100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38510,6 +38510,24 @@
       </c>
       <c r="D2099" t="inlineStr"/>
     </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr">
+        <is>
+          <t>Product formulation issue</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2100" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Circumstance or information capable of leading to medication error
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2100"/>
+  <dimension ref="A1:D2101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38528,6 +38528,24 @@
       </c>
       <c r="D2100" t="inlineStr"/>
     </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>Circumstance or information capable of leading to medication error</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2101" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Treatment noncompliance
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2101"/>
+  <dimension ref="A1:D2102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38546,6 +38546,24 @@
       </c>
       <c r="D2101" t="inlineStr"/>
     </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr">
+        <is>
+          <t>Treatment noncompliance</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2102" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: RIVAROXABAN / Urine analysis abnormal
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2102"/>
+  <dimension ref="A1:D2103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38564,6 +38564,24 @@
       </c>
       <c r="D2102" t="inlineStr"/>
     </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>RIVAROXABAN</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>Urine analysis abnormal</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2103" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: APREMILAST / Skin injury
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2103"/>
+  <dimension ref="A1:D2104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38582,6 +38582,24 @@
       </c>
       <c r="D2103" t="inlineStr"/>
     </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr">
+        <is>
+          <t>APREMILAST</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr">
+        <is>
+          <t>Skin injury</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2104" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Urethritis noninfective
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2104"/>
+  <dimension ref="A1:D2105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38600,6 +38600,24 @@
       </c>
       <c r="D2104" t="inlineStr"/>
     </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>Urethritis noninfective</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2105" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Squamous cell carcinoma
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2105"/>
+  <dimension ref="A1:D2106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38618,6 +38618,24 @@
       </c>
       <c r="D2105" t="inlineStr"/>
     </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr">
+        <is>
+          <t>Squamous cell carcinoma</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2106" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Diabetic ketosis
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2106"/>
+  <dimension ref="A1:D2107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38636,6 +38636,24 @@
       </c>
       <c r="D2106" t="inlineStr"/>
     </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>Diabetic ketosis</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2107" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ICATIBANT / Swelling face
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2107"/>
+  <dimension ref="A1:D2108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38654,6 +38654,24 @@
       </c>
       <c r="D2107" t="inlineStr"/>
     </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr">
+        <is>
+          <t>ICATIBANT</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr">
+        <is>
+          <t>Swelling face</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2108" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Gingival pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2108"/>
+  <dimension ref="A1:D2109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38672,6 +38672,24 @@
       </c>
       <c r="D2108" t="inlineStr"/>
     </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>Gingival pain</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2109" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Glossodynia
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2109"/>
+  <dimension ref="A1:D2110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38690,6 +38690,24 @@
       </c>
       <c r="D2109" t="inlineStr"/>
     </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr">
+        <is>
+          <t>Glossodynia</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2110" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Infection
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2110"/>
+  <dimension ref="A1:D2111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38708,6 +38708,24 @@
       </c>
       <c r="D2110" t="inlineStr"/>
     </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>Infection</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2111" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Renal disorder
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2111"/>
+  <dimension ref="A1:D2112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38726,6 +38726,24 @@
       </c>
       <c r="D2111" t="inlineStr"/>
     </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr">
+        <is>
+          <t>Renal disorder</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2112" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Liver disorder
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2112"/>
+  <dimension ref="A1:D2113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38744,6 +38744,24 @@
       </c>
       <c r="D2112" t="inlineStr"/>
     </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>Liver disorder</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2113" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Blood urine present
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2113"/>
+  <dimension ref="A1:D2114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38762,6 +38762,24 @@
       </c>
       <c r="D2113" t="inlineStr"/>
     </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr">
+        <is>
+          <t>Blood urine present</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D2114" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Antipsychotic drug level
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2114"/>
+  <dimension ref="A1:D2115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38780,6 +38780,24 @@
       </c>
       <c r="D2114" t="inlineStr"/>
     </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>Antipsychotic drug level</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2115" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Gastrointestinal pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2115"/>
+  <dimension ref="A1:D2116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38798,6 +38798,24 @@
       </c>
       <c r="D2115" t="inlineStr"/>
     </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr">
+        <is>
+          <t>Gastrointestinal pain</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2116" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Anal fistula
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2116"/>
+  <dimension ref="A1:D2117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38816,6 +38816,24 @@
       </c>
       <c r="D2116" t="inlineStr"/>
     </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>Anal fistula</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2117" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: ABIRATERONE / Oral pain
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2117"/>
+  <dimension ref="A1:D2118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38834,6 +38834,24 @@
       </c>
       <c r="D2117" t="inlineStr"/>
     </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr">
+        <is>
+          <t>ABIRATERONE</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr">
+        <is>
+          <t>Oral pain</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2118" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Foot operation
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2118"/>
+  <dimension ref="A1:D2119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38852,6 +38852,24 @@
       </c>
       <c r="D2118" t="inlineStr"/>
     </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>Foot operation</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2119" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Lower urinary tract symptoms
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2119"/>
+  <dimension ref="A1:D2120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38870,6 +38870,24 @@
       </c>
       <c r="D2119" t="inlineStr"/>
     </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr">
+        <is>
+          <t>Lower urinary tract symptoms</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2120" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Hypotension
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2120"/>
+  <dimension ref="A1:D2121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38888,6 +38888,24 @@
       </c>
       <c r="D2120" t="inlineStr"/>
     </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>Hypotension</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2121" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Affective disorder
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2121"/>
+  <dimension ref="A1:D2122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38906,6 +38906,24 @@
       </c>
       <c r="D2121" t="inlineStr"/>
     </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr">
+        <is>
+          <t>Affective disorder</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2122" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: PIRFENIDONE / Aggression
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2122"/>
+  <dimension ref="A1:D2123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38924,6 +38924,24 @@
       </c>
       <c r="D2122" t="inlineStr"/>
     </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>PIRFENIDONE</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>Aggression</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2123" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Urine analysis abnormal
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2123"/>
+  <dimension ref="A1:D2124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38942,6 +38942,24 @@
       </c>
       <c r="D2123" t="inlineStr"/>
     </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr">
+        <is>
+          <t>Urine analysis abnormal</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2124" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: DAPAGLIFLOZIN / Perineal abscess
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2124"/>
+  <dimension ref="A1:D2125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38960,6 +38960,28 @@
       </c>
       <c r="D2124" t="inlineStr"/>
     </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>DAPAGLIFLOZIN</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>Perineal abscess</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2125" t="inlineStr">
+        <is>
+          <t>Listed with Fournier’s gangrene</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update listedness: NINTEDANIB / Pollakiuria
</commit_message>
<xml_diff>
--- a/data/Listedness_CX.xlsx
+++ b/data/Listedness_CX.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2125"/>
+  <dimension ref="A1:D2126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38982,6 +38982,24 @@
         </is>
       </c>
     </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr">
+        <is>
+          <t>NINTEDANIB</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr">
+        <is>
+          <t>Pollakiuria</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr">
+        <is>
+          <t>Unexpected</t>
+        </is>
+      </c>
+      <c r="D2126" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>